<commit_message>
1. update color scheme
</commit_message>
<xml_diff>
--- a/report_template/chart_export.xlsx
+++ b/report_template/chart_export.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\webApp\Datalogger2\report_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repo\Datalogger2\report_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6DCB74A-3B30-4CF2-8E05-B5348A7304EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1408C135-BA38-4DF7-AE6D-973C1177CBDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
+    <sheet name="工作表2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -22,6 +23,23 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>校正</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>保養</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>無效</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -46,15 +64,33 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCEEFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC4E1FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD2D2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,17 +98,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -81,6 +141,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFD2D2"/>
+      <color rgb="FFC4E1FF"/>
+      <color rgb="FFCEEFCE"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -356,7 +423,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="20" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="20" defaultRowHeight="16.75" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="16384" width="20" style="1"/>
   </cols>
@@ -365,4 +432,26 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97EF769-9E0F-4986-B107-9977F6EE1AE5}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="16.75" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>